<commit_message>
update 2014 majoritarian IDs for cands, and associated loaders
</commit_message>
<xml_diff>
--- a/src/data/downloads/local_2014_2014_oct_sakrebulo_by_election_20141020_data.xlsx
+++ b/src/data/downloads/local_2014_2014_oct_sakrebulo_by_election_20141020_data.xlsx
@@ -146,7 +146,7 @@
     <t>File Generated</t>
   </si>
   <si>
-    <t>2026-05-25T13:08:48.807Z</t>
+    <t>2026-06-13T11:36:45.147Z</t>
   </si>
   <si>
     <t>Data Source</t>
@@ -867,7 +867,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
@@ -1063,7 +1063,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
@@ -1355,7 +1355,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
@@ -1551,7 +1551,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>